<commit_message>
auto: sync reports 2026-05-05 15:51
</commit_message>
<xml_diff>
--- a/feedback-reports/Building_Agentic_AI_Systems.xlsx
+++ b/feedback-reports/Building_Agentic_AI_Systems.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandita.vora\OneDrive - NIIT Limited\NIIT-AI Powered FSE - General\Design Docs\FSE-v6\Website-Feedback\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandita.vora\OneDrive - NIIT Limited\NIIT-AI Powered FSE - General\Design Docs\FSE-v6\Feedback-App\feedback-reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="187" documentId="11_7AC81A541246E63F6F55F8144F5DCE3A17456C52" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB49CF54-B913-462F-9C2C-7A4F66A9B270}"/>
+  <xr:revisionPtr revIDLastSave="199" documentId="11_7AC81A541246E63F6F55F8144F5DCE3A17456C52" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{172547A3-32CF-42E3-829A-F2072F975594}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,23 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="71">
   <si>
     <t>Program Name:</t>
   </si>
@@ -120,6 +109,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> SLO-Driven Agentic System Design
 </t>
@@ -129,6 +119,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>Design real-world, scalable agentic systems with clear architecture and decision frameworks.
 •</t>
@@ -139,6 +130,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> Autonomous Systems in Action
 </t>
@@ -148,6 +140,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>Build and iterate intelligent agents using RAG, tools, and multi-agent workflows.
 •</t>
@@ -158,6 +151,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> Production-Ready Delivery
 </t>
@@ -167,6 +161,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>Validate with observability, security, and performance testing, ending in a final demo and runbook.</t>
     </r>
@@ -222,6 +217,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Replace with:
@@ -233,6 +229,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Core Python &amp; Data Foundations
@@ -243,6 +240,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Build strong fundamentals with Python structures, functions, modular code, and structured data models.
@@ -254,6 +252,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">API Development &amp; LLM Integration
@@ -264,6 +263,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Develop robust REST APIs, handle I/O and validation, and integrate LLM APIs into applications.
@@ -275,6 +275,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Testing, Real-Time Systems &amp; AI Acceleration
@@ -285,6 +286,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Ensure reliability with testing, enable real-time communication, and leverage GenAI for code, docs, and optimization.</t>
@@ -302,6 +304,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Replace with below content:
@@ -313,6 +316,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">End-to-End RAG Pipeline
@@ -323,6 +327,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Build ingestion, chunking, embedding, and hybrid retrieval with grounded, citation-backed responses.
@@ -334,6 +339,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Secure &amp; Tool-Integrated Retrieval
@@ -344,6 +350,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Apply guardrails, PII protection, and integrate MCP tools to connect real backend systems.
@@ -355,6 +362,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Memory, Handoff &amp; SLO Validation
@@ -365,6 +373,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Enable memory and human handoff, and validate performance against accuracy and latency SLOs.</t>
@@ -418,6 +427,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Replace the entire content with the below one:
 1. </t>
@@ -428,6 +438,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Wellbeing Coach – Your Personalized 5-Minute Mental Booster
 </t>
@@ -437,6 +448,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 An AI-powered application that understands user input and context to deliver personalized wellness activities, providing quick and effective interventions through intelligent recommendations and adaptive responses.
@@ -449,6 +461,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Real Estate Assistant – AI-Powered Home Search Companion
 </t>
@@ -458,6 +471,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 A conversational AI agent that helps users discover, compare, and evaluate homes through personalized, context-aware interactions, integrating tools, memory, and workflows to deliver relevant property insights.
@@ -470,6 +484,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> MedLearn Assistant – AI-Powered Medical Education Companion
 </t>
@@ -479,6 +494,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t>An agentic RAG system that processes medical textbooks and multi-modal content to deliver accurate, explainable answers for learning and concept clarification.
 Tags: GENAI, RAG, MULTI-MODAL, DATABASE, AI SECURITY
@@ -490,6 +506,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> Autonomous Social Media Content Studio – Multi-Agent Publishing System
 </t>
@@ -499,6 +516,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 A multi-agent system that transforms a single idea into platform-specific content, using specialized agents, review loops, and coordinated workflows to deliver consistent, publish-ready outputs.
@@ -511,6 +529,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">Multi-Agent Retail Policy Intelligence System
 </t>
@@ -520,6 +539,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 A crew of agents that interprets retail policies, validates decisions against business rules, and provides consistent, explainable outcomes for policy-driven scenarios across operations.
@@ -532,6 +552,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> Multi-Agent Support Resolution System with Human in the Loop
 </t>
@@ -541,6 +562,7 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve">
 A hierarchical workflow of agents with Support Specialist and Resolution QA roles that diagnose issues using documentation and historical data, escalating unresolved or high-risk cases to human experts.
@@ -588,12 +610,21 @@
   <si>
     <t>Replace with: '25+ Tools &amp; Frameworks'</t>
   </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>suggestion is fixed</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -606,34 +637,40 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -655,6 +692,7 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -676,6 +714,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -698,7 +737,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -721,12 +760,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -767,6 +826,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1072,20 +1140,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="80" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="45.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="45.5546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="40" customWidth="1"/>
     <col min="6" max="6" width="45" customWidth="1"/>
     <col min="7" max="7" width="63" customWidth="1"/>
-    <col min="8" max="8" width="40.7109375" customWidth="1"/>
+    <col min="8" max="8" width="40.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="6" customFormat="1" ht="36.75" customHeight="1">
+    <row r="1" spans="1:8" s="6" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1102,8 +1170,9 @@
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
-    </row>
-    <row r="2" spans="1:7" s="6" customFormat="1" ht="36.75" customHeight="1">
+      <c r="H1" s="4"/>
+    </row>
+    <row r="2" spans="1:8" s="6" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -1115,8 +1184,9 @@
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="H2" s="4"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -1136,10 +1206,13 @@
         <v>10</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="H3" s="16" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="72">
+    <row r="4" spans="1:8" ht="69" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>1</v>
       </c>
@@ -1156,8 +1229,14 @@
       <c r="F4" s="9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="15">
+      <c r="G4" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
         <v>2</v>
       </c>
@@ -1175,8 +1254,9 @@
         <v>19</v>
       </c>
       <c r="G5" s="10"/>
-    </row>
-    <row r="6" spans="1:7" ht="187.15">
+      <c r="H5" s="18"/>
+    </row>
+    <row r="6" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>3</v>
       </c>
@@ -1196,7 +1276,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="28.5">
+    <row r="7" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A7" s="13">
         <v>4</v>
       </c>
@@ -1216,7 +1296,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="28.5">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>5</v>
       </c>
@@ -1234,7 +1314,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="275.25">
+    <row r="9" spans="1:8" ht="262.2" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
         <v>6</v>
       </c>
@@ -1252,7 +1332,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="28.5">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>7</v>
       </c>
@@ -1270,7 +1350,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="267" customHeight="1">
+    <row r="11" spans="1:8" ht="267" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
         <v>8</v>
       </c>
@@ -1288,7 +1368,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="198">
+    <row r="12" spans="1:8" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>9</v>
       </c>
@@ -1306,7 +1386,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="28.5">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="13">
         <v>10</v>
       </c>
@@ -1324,7 +1404,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="28.5">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>11</v>
       </c>
@@ -1342,7 +1422,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="115.5">
+    <row r="15" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
       <c r="A15" s="13">
         <v>12</v>
       </c>
@@ -1362,7 +1442,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="57.75">
+    <row r="16" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>13</v>
       </c>
@@ -1382,7 +1462,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="409.6">
+    <row r="17" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A17" s="13">
         <v>14</v>
       </c>
@@ -1400,7 +1480,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="86.25">
+    <row r="18" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>15</v>
       </c>
@@ -1418,7 +1498,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="381.75">
+    <row r="19" spans="1:8" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A19" s="13">
         <v>16</v>
       </c>
@@ -1439,7 +1519,7 @@
       </c>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" ht="41.45">
+    <row r="20" spans="1:8" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>17</v>
       </c>
@@ -1459,8 +1539,6 @@
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15"/>
-    <row r="22" spans="1:8" ht="15"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{223444A8-3458-4270-B4E5-AA1FE6ABB98E}"/>
@@ -1470,12 +1548,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008081BF50E816F94B87E854E2907183B0" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f6f57204d0cc9b1c65f7ab94eaa7dcc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8b8ad293-1655-4b1e-95cd-578b981aff66" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0ed196dee19b1527225c6137bc92e865" ns2:_="">
     <xsd:import namespace="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
@@ -1637,6 +1709,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1647,13 +1725,43 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90732CA2-C0B0-4DE0-9AA4-0FF18513580E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0ACE443-5E35-4A80-AAC5-EB300BF92F41}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C0ACE443-5E35-4A80-AAC5-EB300BF92F41}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90732CA2-C0B0-4DE0-9AA4-0FF18513580E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A79093BA-E29B-4EFA-AAD0-EE916A07E6C2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A79093BA-E29B-4EFA-AAD0-EE916A07E6C2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
auto: sync reports 2026-05-05 15:55
</commit_message>
<xml_diff>
--- a/feedback-reports/Building_Agentic_AI_Systems.xlsx
+++ b/feedback-reports/Building_Agentic_AI_Systems.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandita.vora\OneDrive - NIIT Limited\NIIT-AI Powered FSE - General\Design Docs\FSE-v6\Feedback-App\feedback-reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="11_7AC81A541246E63F6F55F8144F5DCE3A17456C52" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{172547A3-32CF-42E3-829A-F2072F975594}"/>
+  <xr:revisionPtr revIDLastSave="200" documentId="11_7AC81A541246E63F6F55F8144F5DCE3A17456C52" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{931D2F2B-4048-4F53-8815-8DBA3BC7B58D}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="69">
   <si>
     <t>Program Name:</t>
   </si>
@@ -612,12 +612,6 @@
   </si>
   <si>
     <t>Status</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>suggestion is fixed</t>
   </si>
 </sst>
 </file>
@@ -1229,12 +1223,8 @@
       <c r="F4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="H4" s="17" t="s">
-        <v>70</v>
-      </c>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
@@ -1710,18 +1700,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1743,25 +1733,25 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90732CA2-C0B0-4DE0-9AA4-0FF18513580E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A79093BA-E29B-4EFA-AAD0-EE916A07E6C2}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A79093BA-E29B-4EFA-AAD0-EE916A07E6C2}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90732CA2-C0B0-4DE0-9AA4-0FF18513580E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
auto: sync reports from external folder 2026-05-05 16:06
</commit_message>
<xml_diff>
--- a/feedback-reports/Building_Agentic_AI_Systems.xlsx
+++ b/feedback-reports/Building_Agentic_AI_Systems.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandita.vora\OneDrive - NIIT Limited\NIIT-AI Powered FSE - General\Design Docs\FSE-v6\Feedback-App\feedback-reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandita.vora\OneDrive - NIIT Limited\NIIT-AI Powered FSE - General\Design Docs\FSE-v6\Website-Feedback\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="200" documentId="11_7AC81A541246E63F6F55F8144F5DCE3A17456C52" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{931D2F2B-4048-4F53-8815-8DBA3BC7B58D}"/>
+  <xr:revisionPtr revIDLastSave="196" documentId="11_7AC81A541246E63F6F55F8144F5DCE3A17456C52" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{17162C25-8138-403F-A7FD-6785D7C11C20}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="71">
   <si>
     <t>Program Name:</t>
   </si>
@@ -60,6 +60,9 @@
     <t>Fix Suggested</t>
   </si>
   <si>
+    <t>Status</t>
+  </si>
+  <si>
     <t>Remarks</t>
   </si>
   <si>
@@ -73,6 +76,9 @@
   </si>
   <si>
     <t>Replace with: 'Agents for Every Ambition – a premium learning initiative by NIIT, building job-ready AI leaders with industry-driven training, real-world expertise, and in-demand artificial intelligence skills.'</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
   <si>
     <t>Program Overview</t>
@@ -611,7 +617,7 @@
     <t>Replace with: '25+ Tools &amp; Frameworks'</t>
   </si>
   <si>
-    <t>Status</t>
+    <t>suggestion is implemented and fixed</t>
   </si>
 </sst>
 </file>
@@ -731,7 +737,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -754,32 +760,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFBFBFBF"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -820,15 +806,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1200,10 +1177,10 @@
         <v>10</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H3" s="16" t="s">
         <v>11</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="69" x14ac:dyDescent="0.3">
@@ -1211,59 +1188,62 @@
         <v>1</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E4" s="9"/>
       <c r="F4" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="17"/>
-      <c r="H4" s="17"/>
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
         <v>2</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="14" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G5" s="10"/>
-      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>3</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="27.6" x14ac:dyDescent="0.3">
@@ -1271,19 +1251,19 @@
         <v>4</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -1291,17 +1271,17 @@
         <v>5</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E8" s="9"/>
       <c r="F8" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="262.2" x14ac:dyDescent="0.3">
@@ -1309,17 +1289,17 @@
         <v>6</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E9" s="9"/>
       <c r="F9" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -1327,17 +1307,17 @@
         <v>7</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E10" s="9"/>
       <c r="F10" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="267" customHeight="1" x14ac:dyDescent="0.3">
@@ -1345,17 +1325,17 @@
         <v>8</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E11" s="9"/>
       <c r="F11" s="12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="172.8" x14ac:dyDescent="0.3">
@@ -1363,17 +1343,17 @@
         <v>9</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="12" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -1381,17 +1361,17 @@
         <v>10</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -1399,17 +1379,17 @@
         <v>11</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="110.4" x14ac:dyDescent="0.3">
@@ -1417,19 +1397,19 @@
         <v>12</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="55.2" x14ac:dyDescent="0.3">
@@ -1437,19 +1417,19 @@
         <v>13</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
@@ -1457,17 +1437,17 @@
         <v>14</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="11" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="82.8" x14ac:dyDescent="0.3">
@@ -1475,17 +1455,17 @@
         <v>15</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="345.6" x14ac:dyDescent="0.3">
@@ -1493,19 +1473,19 @@
         <v>16</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H19" s="2"/>
     </row>
@@ -1514,19 +1494,19 @@
         <v>17</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1700,18 +1680,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1733,25 +1713,25 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90732CA2-C0B0-4DE0-9AA4-0FF18513580E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A79093BA-E29B-4EFA-AAD0-EE916A07E6C2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90732CA2-C0B0-4DE0-9AA4-0FF18513580E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="8b8ad293-1655-4b1e-95cd-578b981aff66"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>